<commit_message>
Actualizacion de los sprints
</commit_message>
<xml_diff>
--- a/Documentacion Sprint (01 - 11)/Sprint 1 documentacion/Sprint_01_Backlog_ICARO.xlsx
+++ b/Documentacion Sprint (01 - 11)/Sprint 1 documentacion/Sprint_01_Backlog_ICARO.xlsx
@@ -1,29 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hp\Desktop\Sistema_Gestion_Integral_Constructora\Documentos Base\Sprint 1 documentacion\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hp\Desktop\Sistema_Gestion_Integral_Constructora\Documentacion Sprint (01 - 11)\Sprint 1 documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B279D708-B4C9-4561-8E28-25A4FAE02988}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6147AE27-A84D-4973-9CB8-D6C51001117A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5415" yWindow="1125" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog Sprint 01" sheetId="1" r:id="rId1"/>
-    <sheet name="Resumen Velocidad" sheetId="2" r:id="rId2"/>
-    <sheet name="Glosario" sheetId="3" r:id="rId3"/>
-    <sheet name="Resumen de Casos de Prueba " sheetId="4" r:id="rId4"/>
+    <sheet name="Resumen de Casos de Prueba " sheetId="4" r:id="rId2"/>
+    <sheet name="Resumen Velocidad" sheetId="2" r:id="rId3"/>
+    <sheet name="Glosario" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="212">
   <si>
     <t>SPRINT BACKLOG — Sprint 01: Infraestructura Base, Autenticación y Gestión de Usuarios</t>
   </si>
@@ -656,13 +656,16 @@
   </si>
   <si>
     <t>security.test.js – Test 15</t>
+  </si>
+  <si>
+    <t>Los estados presentados en este documento corresponden al estado del Product/Sprint Backlog al cierre del Sprint respectivo. Debido a la naturaleza iterativa e incremental del proyecto, los elementos identificados como pendientes, diferidos o parcialmente implementados pudieron ser desarrollados y completados en sprints posteriores. Para conocer el estado definitivo de cada historia de usuario o historia técnica, debe consultarse el Product Backlog Consolidado al cierre del proyecto.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -755,8 +758,22 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -793,8 +810,13 @@
         <fgColor rgb="FF2E75B6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -871,11 +893,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -961,6 +999,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="6" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -998,8 +1039,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Notas" xfId="1" builtinId="10"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1299,7 +1341,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1317,124 +1359,124 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="33"/>
-      <c r="I1" s="33"/>
-      <c r="J1" s="33"/>
-      <c r="K1" s="33"/>
-      <c r="L1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
+      <c r="J1" s="34"/>
+      <c r="K1" s="34"/>
+      <c r="L1" s="34"/>
     </row>
     <row r="2" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="41" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="33"/>
-      <c r="G2" s="33"/>
-      <c r="H2" s="33"/>
-      <c r="I2" s="33"/>
-      <c r="J2" s="33"/>
-      <c r="K2" s="33"/>
-      <c r="L2" s="33"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
+      <c r="I2" s="34"/>
+      <c r="J2" s="34"/>
+      <c r="K2" s="34"/>
+      <c r="L2" s="34"/>
     </row>
     <row r="3" spans="1:12" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="34" t="s">
+      <c r="B3" s="35" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="35"/>
-      <c r="D3" s="35"/>
-      <c r="E3" s="35"/>
-      <c r="F3" s="36"/>
+      <c r="C3" s="36"/>
+      <c r="D3" s="36"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="37"/>
       <c r="G3" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="34" t="s">
+      <c r="H3" s="35" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="35"/>
-      <c r="J3" s="35"/>
-      <c r="K3" s="35"/>
-      <c r="L3" s="36"/>
+      <c r="I3" s="36"/>
+      <c r="J3" s="36"/>
+      <c r="K3" s="36"/>
+      <c r="L3" s="37"/>
     </row>
     <row r="4" spans="1:12" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="37">
+      <c r="B4" s="38">
         <v>46125</v>
       </c>
-      <c r="C4" s="38"/>
-      <c r="D4" s="38"/>
-      <c r="E4" s="38"/>
-      <c r="F4" s="39"/>
+      <c r="C4" s="39"/>
+      <c r="D4" s="39"/>
+      <c r="E4" s="39"/>
+      <c r="F4" s="40"/>
       <c r="G4" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="H4" s="37">
+      <c r="H4" s="38">
         <v>46129</v>
       </c>
-      <c r="I4" s="38"/>
-      <c r="J4" s="38"/>
-      <c r="K4" s="38"/>
-      <c r="L4" s="39"/>
+      <c r="I4" s="39"/>
+      <c r="J4" s="39"/>
+      <c r="K4" s="39"/>
+      <c r="L4" s="40"/>
     </row>
     <row r="5" spans="1:12" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="34" t="s">
+      <c r="B5" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="35"/>
-      <c r="D5" s="35"/>
-      <c r="E5" s="35"/>
-      <c r="F5" s="36"/>
+      <c r="C5" s="36"/>
+      <c r="D5" s="36"/>
+      <c r="E5" s="36"/>
+      <c r="F5" s="37"/>
       <c r="G5" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="H5" s="34" t="s">
+      <c r="H5" s="35" t="s">
         <v>110</v>
       </c>
-      <c r="I5" s="35"/>
-      <c r="J5" s="35"/>
-      <c r="K5" s="35"/>
-      <c r="L5" s="36"/>
+      <c r="I5" s="36"/>
+      <c r="J5" s="36"/>
+      <c r="K5" s="36"/>
+      <c r="L5" s="37"/>
     </row>
     <row r="6" spans="1:12" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="34" t="s">
+      <c r="B6" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="35"/>
-      <c r="D6" s="35"/>
-      <c r="E6" s="35"/>
-      <c r="F6" s="36"/>
+      <c r="C6" s="36"/>
+      <c r="D6" s="36"/>
+      <c r="E6" s="36"/>
+      <c r="F6" s="37"/>
       <c r="G6" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="34" t="s">
+      <c r="H6" s="35" t="s">
         <v>14</v>
       </c>
-      <c r="I6" s="35"/>
-      <c r="J6" s="35"/>
-      <c r="K6" s="35"/>
-      <c r="L6" s="36"/>
+      <c r="I6" s="36"/>
+      <c r="J6" s="36"/>
+      <c r="K6" s="36"/>
+      <c r="L6" s="37"/>
     </row>
     <row r="7" spans="1:12" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
@@ -1741,13 +1783,13 @@
       </c>
     </row>
     <row r="15" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="30" t="s">
+      <c r="A15" s="31" t="s">
         <v>74</v>
       </c>
-      <c r="B15" s="31"/>
-      <c r="C15" s="31"/>
-      <c r="D15" s="31"/>
-      <c r="E15" s="31"/>
+      <c r="B15" s="32"/>
+      <c r="C15" s="32"/>
+      <c r="D15" s="32"/>
+      <c r="E15" s="32"/>
       <c r="F15" s="8">
         <v>34</v>
       </c>
@@ -1760,8 +1802,53 @@
       <c r="K15" s="7"/>
       <c r="L15" s="7"/>
     </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="30" t="s">
+        <v>211</v>
+      </c>
+      <c r="B17" s="30"/>
+      <c r="C17" s="30"/>
+      <c r="D17" s="30"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="30"/>
+      <c r="B18" s="30"/>
+      <c r="C18" s="30"/>
+      <c r="D18" s="30"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="30"/>
+      <c r="B19" s="30"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="30"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="30"/>
+      <c r="B20" s="30"/>
+      <c r="C20" s="30"/>
+      <c r="D20" s="30"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="30"/>
+      <c r="B21" s="30"/>
+      <c r="C21" s="30"/>
+      <c r="D21" s="30"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="30"/>
+      <c r="B22" s="30"/>
+      <c r="C22" s="30"/>
+      <c r="D22" s="30"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="30"/>
+      <c r="B23" s="30"/>
+      <c r="C23" s="30"/>
+      <c r="D23" s="30"/>
+    </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="12">
+    <mergeCell ref="A17:D23"/>
     <mergeCell ref="A15:E15"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="B3:F3"/>
@@ -1779,403 +1866,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="38" customWidth="1"/>
-    <col min="2" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="22" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="41" t="s">
-        <v>75</v>
-      </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="B2" s="23" t="s">
-        <v>77</v>
-      </c>
-      <c r="C2" s="23" t="s">
-        <v>78</v>
-      </c>
-      <c r="D2" s="23" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="B3" s="25">
-        <v>34</v>
-      </c>
-      <c r="C3" s="25">
-        <v>34</v>
-      </c>
-      <c r="D3" s="26" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="27" t="s">
-        <v>82</v>
-      </c>
-      <c r="B4" s="28">
-        <v>3</v>
-      </c>
-      <c r="C4" s="28">
-        <v>3</v>
-      </c>
-      <c r="D4" s="29" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="24" t="s">
-        <v>84</v>
-      </c>
-      <c r="B5" s="25">
-        <v>4</v>
-      </c>
-      <c r="C5" s="25">
-        <v>4</v>
-      </c>
-      <c r="D5" s="26" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="27" t="s">
-        <v>86</v>
-      </c>
-      <c r="B6" s="28">
-        <v>7</v>
-      </c>
-      <c r="C6" s="28">
-        <v>7</v>
-      </c>
-      <c r="D6" s="29" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="24" t="s">
-        <v>88</v>
-      </c>
-      <c r="B7" s="25">
-        <v>7</v>
-      </c>
-      <c r="C7" s="25">
-        <v>7</v>
-      </c>
-      <c r="D7" s="26" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="27" t="s">
-        <v>90</v>
-      </c>
-      <c r="B8" s="28">
-        <v>0</v>
-      </c>
-      <c r="C8" s="28">
-        <v>0</v>
-      </c>
-      <c r="D8" s="29" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="24" t="s">
-        <v>92</v>
-      </c>
-      <c r="B9" s="25">
-        <v>0</v>
-      </c>
-      <c r="C9" s="25">
-        <v>0</v>
-      </c>
-      <c r="D9" s="26" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="27" t="s">
-        <v>94</v>
-      </c>
-      <c r="B10" s="28">
-        <v>17</v>
-      </c>
-      <c r="C10" s="28">
-        <v>17</v>
-      </c>
-      <c r="D10" s="29" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="24" t="s">
-        <v>95</v>
-      </c>
-      <c r="B11" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="C11" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="D11" s="26" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="27" t="s">
-        <v>97</v>
-      </c>
-      <c r="B12" s="28">
-        <v>15</v>
-      </c>
-      <c r="C12" s="28">
-        <v>15</v>
-      </c>
-      <c r="D12" s="29" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="24" t="s">
-        <v>99</v>
-      </c>
-      <c r="B13" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="C13" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="D13" s="26" t="s">
-        <v>100</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{763E11AF-F722-4524-841D-EB284C50087B}">
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="11.42578125" customWidth="1"/>
-    <col min="2" max="2" width="29.85546875" customWidth="1"/>
-    <col min="3" max="3" width="42.85546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="43" t="s">
-        <v>113</v>
-      </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>102</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="B3" s="12" t="s">
-        <v>115</v>
-      </c>
-      <c r="C3" s="12" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="B4" s="14" t="s">
-        <v>117</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="11" t="s">
-        <v>103</v>
-      </c>
-      <c r="B5" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
-        <v>104</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>121</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="B7" s="12" t="s">
-        <v>123</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="13" t="s">
-        <v>107</v>
-      </c>
-      <c r="B8" s="14" t="s">
-        <v>125</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="11" t="s">
-        <v>127</v>
-      </c>
-      <c r="B9" s="12" t="s">
-        <v>128</v>
-      </c>
-      <c r="C9" s="12" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="13" t="s">
-        <v>130</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="B11" s="12" t="s">
-        <v>133</v>
-      </c>
-      <c r="C11" s="12" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="13" t="s">
-        <v>106</v>
-      </c>
-      <c r="B12" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="C12" s="14" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="B13" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="13" t="s">
-        <v>138</v>
-      </c>
-      <c r="B14" s="14" t="s">
-        <v>139</v>
-      </c>
-      <c r="C14" s="14" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="11" t="s">
-        <v>141</v>
-      </c>
-      <c r="B15" s="12" t="s">
-        <v>142</v>
-      </c>
-      <c r="C15" s="12" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="B16" s="14" t="s">
-        <v>145</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="11" t="s">
-        <v>147</v>
-      </c>
-      <c r="B17" s="12" t="s">
-        <v>148</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>149</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
-  </mergeCells>
-  <phoneticPr fontId="12" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1898C963-16D1-41BA-A783-154B1ABEC1D5}">
   <dimension ref="A1:M17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2188,14 +1878,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="45" t="s">
         <v>209</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
@@ -2619,4 +2309,401 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="38" customWidth="1"/>
+    <col min="2" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="42" t="s">
+        <v>75</v>
+      </c>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="23" t="s">
+        <v>76</v>
+      </c>
+      <c r="B2" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="C2" s="23" t="s">
+        <v>78</v>
+      </c>
+      <c r="D2" s="23" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="B3" s="25">
+        <v>34</v>
+      </c>
+      <c r="C3" s="25">
+        <v>34</v>
+      </c>
+      <c r="D3" s="26" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="27" t="s">
+        <v>82</v>
+      </c>
+      <c r="B4" s="28">
+        <v>3</v>
+      </c>
+      <c r="C4" s="28">
+        <v>3</v>
+      </c>
+      <c r="D4" s="29" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="24" t="s">
+        <v>84</v>
+      </c>
+      <c r="B5" s="25">
+        <v>4</v>
+      </c>
+      <c r="C5" s="25">
+        <v>4</v>
+      </c>
+      <c r="D5" s="26" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="27" t="s">
+        <v>86</v>
+      </c>
+      <c r="B6" s="28">
+        <v>7</v>
+      </c>
+      <c r="C6" s="28">
+        <v>7</v>
+      </c>
+      <c r="D6" s="29" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="24" t="s">
+        <v>88</v>
+      </c>
+      <c r="B7" s="25">
+        <v>7</v>
+      </c>
+      <c r="C7" s="25">
+        <v>7</v>
+      </c>
+      <c r="D7" s="26" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="B8" s="28">
+        <v>0</v>
+      </c>
+      <c r="C8" s="28">
+        <v>0</v>
+      </c>
+      <c r="D8" s="29" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="24" t="s">
+        <v>92</v>
+      </c>
+      <c r="B9" s="25">
+        <v>0</v>
+      </c>
+      <c r="C9" s="25">
+        <v>0</v>
+      </c>
+      <c r="D9" s="26" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="27" t="s">
+        <v>94</v>
+      </c>
+      <c r="B10" s="28">
+        <v>17</v>
+      </c>
+      <c r="C10" s="28">
+        <v>17</v>
+      </c>
+      <c r="D10" s="29" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="24" t="s">
+        <v>95</v>
+      </c>
+      <c r="B11" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="C11" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="D11" s="26" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="27" t="s">
+        <v>97</v>
+      </c>
+      <c r="B12" s="28">
+        <v>15</v>
+      </c>
+      <c r="C12" s="28">
+        <v>15</v>
+      </c>
+      <c r="D12" s="29" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="24" t="s">
+        <v>99</v>
+      </c>
+      <c r="B13" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="C13" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="D13" s="26" t="s">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{763E11AF-F722-4524-841D-EB284C50087B}">
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.42578125" customWidth="1"/>
+    <col min="2" max="2" width="29.85546875" customWidth="1"/>
+    <col min="3" max="3" width="42.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="44" t="s">
+        <v>113</v>
+      </c>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>128</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="13" t="s">
+        <v>130</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>149</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <phoneticPr fontId="12" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>